<commit_message>
small change to supplementary table S7
</commit_message>
<xml_diff>
--- a/Supplementary_Table_S7_Statistical_Metrics.xlsx
+++ b/Supplementary_Table_S7_Statistical_Metrics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmorampa/Documents/labnotebook_code/CHAPTER-3-TOOL-BENCHMARK-FINAL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmorampa/Documents/rnamod-tool-benchmark-code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{0E05DAE6-DB66-7647-8657-9AB5A50F4EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{186DF637-9AA8-884B-A095-942A476228A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32000" yWindow="600" windowWidth="32000" windowHeight="33900" xr2:uid="{07C4EE7B-EB21-7342-9145-E684C6947C82}"/>
   </bookViews>
@@ -140,9 +140,6 @@
     <t>95x</t>
   </si>
   <si>
-    <t>1200x</t>
-  </si>
-  <si>
     <t>Tool</t>
   </si>
   <si>
@@ -175,13 +172,16 @@
   <si>
     <t>Overall Call Fraction (OCF)</t>
   </si>
+  <si>
+    <t>Full</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -672,10 +672,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1070,31 +1070,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>42</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -1105,7 +1105,7 @@
         <v>25</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" s="3">
         <v>6.6456080839385298E-2</v>
@@ -1134,7 +1134,7 @@
         <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D3" s="3">
         <v>7.5298070546771803E-2</v>
@@ -1163,7 +1163,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D4" s="2">
         <v>0.16885676392655599</v>
@@ -1192,7 +1192,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D5" s="2">
         <v>0.18347371167129001</v>
@@ -1221,7 +1221,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" s="2">
         <v>0.35346751536316001</v>
@@ -1250,7 +1250,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D7" s="3">
         <v>0.33183578379699202</v>
@@ -1279,7 +1279,7 @@
         <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" s="2">
         <v>0.35920054716942501</v>
@@ -1308,7 +1308,7 @@
         <v>16</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D9" s="2">
         <v>0.40981258649818703</v>
@@ -1337,7 +1337,7 @@
         <v>17</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D10" s="2">
         <v>0.383453756253054</v>
@@ -1366,7 +1366,7 @@
         <v>17</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D11" s="2">
         <v>0.44474931151661701</v>
@@ -1395,7 +1395,7 @@
         <v>18</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D12" s="2">
         <v>0.428657604567943</v>
@@ -1424,7 +1424,7 @@
         <v>18</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2">
         <v>0.46786123765134202</v>
@@ -1453,7 +1453,7 @@
         <v>19</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D14" s="2">
         <v>0.43865260811121698</v>
@@ -1482,7 +1482,7 @@
         <v>19</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15" s="3">
         <v>0.482432489680439</v>
@@ -1511,7 +1511,7 @@
         <v>20</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D16" s="2">
         <v>0.40883651590377901</v>
@@ -1540,7 +1540,7 @@
         <v>20</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D17" s="2">
         <v>0.472971439279392</v>
@@ -1569,7 +1569,7 @@
         <v>21</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D18" s="2">
         <v>0.45742859757353199</v>
@@ -1598,7 +1598,7 @@
         <v>21</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D19" s="2">
         <v>0.46040033258247598</v>
@@ -1627,7 +1627,7 @@
         <v>23</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D20" s="2">
         <v>0.462521975630306</v>
@@ -1656,7 +1656,7 @@
         <v>23</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D21" s="2">
         <v>0.476905511017229</v>
@@ -1685,7 +1685,7 @@
         <v>24</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D22" s="2">
         <v>0.44881155322051702</v>
@@ -1714,7 +1714,7 @@
         <v>24</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D23" s="3">
         <v>0.48608125514634998</v>
@@ -1743,7 +1743,7 @@
         <v>26</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D24" s="2">
         <v>0.50878294088679299</v>
@@ -1772,7 +1772,7 @@
         <v>26</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D25" s="2">
         <v>0.483280428439819</v>
@@ -1801,7 +1801,7 @@
         <v>27</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D26" s="2">
         <v>0.52807300631573295</v>
@@ -1830,7 +1830,7 @@
         <v>27</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D27" s="2">
         <v>0.48849608192027499</v>
@@ -1859,7 +1859,7 @@
         <v>28</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D28" s="3">
         <v>0.53665155931629505</v>
@@ -1888,7 +1888,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D29" s="2">
         <v>0.49257068579137903</v>
@@ -1917,7 +1917,7 @@
         <v>30</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D30" s="2">
         <v>0.54723798944592605</v>
@@ -1946,7 +1946,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D31" s="2">
         <v>0.49284279312283202</v>
@@ -1975,7 +1975,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D32" s="2">
         <v>0.58673918910771905</v>
@@ -2004,7 +2004,7 @@
         <v>31</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D33" s="2">
         <v>0.48355370209799298</v>
@@ -2033,7 +2033,7 @@
         <v>32</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D34" s="2">
         <v>0.57681525233648401</v>
@@ -2062,7 +2062,7 @@
         <v>32</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D35" s="2">
         <v>0.48019589641967803</v>
@@ -2091,7 +2091,7 @@
         <v>33</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D36" s="3">
         <v>0.59326135727460305</v>
@@ -2120,7 +2120,7 @@
         <v>33</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D37" s="2">
         <v>0.48030456619194301</v>
@@ -2149,7 +2149,7 @@
         <v>34</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D38" s="2">
         <v>0.59125364426612803</v>
@@ -2178,7 +2178,7 @@
         <v>34</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D39" s="2">
         <v>0.47838308260301998</v>
@@ -2207,7 +2207,7 @@
         <v>11</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D40" s="2">
         <v>0.61439955102317301</v>
@@ -2236,7 +2236,7 @@
         <v>11</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D41" s="2">
         <v>0.47038775993285198</v>
@@ -2265,7 +2265,7 @@
         <v>13</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D42" s="2">
         <v>0.57098914481701402</v>
@@ -2294,7 +2294,7 @@
         <v>13</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D43" s="2">
         <v>0.46158123267806001</v>
@@ -2323,7 +2323,7 @@
         <v>15</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D44" s="3">
         <v>0.58371062232742499</v>
@@ -2352,7 +2352,7 @@
         <v>15</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D45" s="2">
         <v>0.44817541167637698</v>
@@ -2381,7 +2381,7 @@
         <v>22</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D46" s="2">
         <v>0.58289338958737202</v>
@@ -2410,7 +2410,7 @@
         <v>22</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D47" s="2">
         <v>0.45382729043916198</v>
@@ -2439,7 +2439,7 @@
         <v>29</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D48" s="2">
         <v>0.56871063643209996</v>
@@ -2468,7 +2468,7 @@
         <v>29</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D49" s="2">
         <v>0.45418707331368902</v>
@@ -2497,7 +2497,7 @@
         <v>0</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D50" s="2">
         <v>0.535856077520525</v>
@@ -2526,7 +2526,7 @@
         <v>0</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D51" s="2">
         <v>0.45956649623603202</v>
@@ -2552,10 +2552,10 @@
         <v>1</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D52" s="2">
         <v>0.469856105734136</v>
@@ -2581,10 +2581,10 @@
         <v>1</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D53" s="2">
         <v>0.43189341657604002</v>
@@ -2613,7 +2613,7 @@
         <v>14</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D54" s="3">
         <v>6.80922865013774E-2</v>
@@ -2638,7 +2638,7 @@
         <v>16</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D55" s="2">
         <v>0.101138659320477</v>
@@ -2667,7 +2667,7 @@
         <v>17</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D56" s="3">
         <v>9.7394175215186896E-2</v>
@@ -2692,7 +2692,7 @@
         <v>17</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D57" s="2">
         <v>0.114357208448117</v>
@@ -2721,7 +2721,7 @@
         <v>18</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D58" s="3">
         <v>7.1335927367054998E-3</v>
@@ -2746,7 +2746,7 @@
         <v>18</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D59" s="2">
         <v>0.161084874721238</v>
@@ -2775,7 +2775,7 @@
         <v>19</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D60" s="3">
         <v>5.2263883975946203E-2</v>
@@ -2804,7 +2804,7 @@
         <v>19</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D61" s="2">
         <v>0.18718142463597001</v>
@@ -2833,7 +2833,7 @@
         <v>20</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D62" s="3">
         <v>5.2263883975946203E-2</v>
@@ -2862,7 +2862,7 @@
         <v>20</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D63" s="2">
         <v>0.22795395513577299</v>
@@ -2891,7 +2891,7 @@
         <v>21</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D64" s="3">
         <v>2.1960853672915899E-2</v>
@@ -2920,7 +2920,7 @@
         <v>21</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D65" s="2">
         <v>0.22676876995058801</v>
@@ -2949,7 +2949,7 @@
         <v>23</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D66" s="3">
         <v>5.1939629760641398E-2</v>
@@ -2978,7 +2978,7 @@
         <v>23</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D67" s="2">
         <v>0.244575276575276</v>
@@ -3007,7 +3007,7 @@
         <v>24</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D68" s="3">
         <v>7.1709311008921903E-2</v>
@@ -3036,7 +3036,7 @@
         <v>24</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D69" s="2">
         <v>0.29180012243648601</v>
@@ -3065,7 +3065,7 @@
         <v>26</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D70" s="3">
         <v>7.6759816059426902E-2</v>
@@ -3094,7 +3094,7 @@
         <v>26</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D71" s="2">
         <v>0.32686968923332499</v>
@@ -3123,7 +3123,7 @@
         <v>27</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D72" s="3">
         <v>8.6500356539267007E-2</v>
@@ -3152,7 +3152,7 @@
         <v>27</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D73" s="2">
         <v>0.35138004756186503</v>
@@ -3181,7 +3181,7 @@
         <v>28</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D74" s="2">
         <v>0.16211419363170301</v>
@@ -3210,7 +3210,7 @@
         <v>28</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D75" s="2">
         <v>0.36534895743986601</v>
@@ -3239,7 +3239,7 @@
         <v>30</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D76" s="2">
         <v>0.17026687104508101</v>
@@ -3268,7 +3268,7 @@
         <v>30</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D77" s="2">
         <v>0.363789886880795</v>
@@ -3297,7 +3297,7 @@
         <v>31</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D78" s="2">
         <v>0.205584892841702</v>
@@ -3326,7 +3326,7 @@
         <v>31</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D79" s="2">
         <v>0.388227716727716</v>
@@ -3355,7 +3355,7 @@
         <v>32</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D80" s="2">
         <v>0.22127781427392301</v>
@@ -3384,7 +3384,7 @@
         <v>32</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D81" s="2">
         <v>0.38454649054648998</v>
@@ -3413,7 +3413,7 @@
         <v>33</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D82" s="2">
         <v>0.195087057343866</v>
@@ -3442,7 +3442,7 @@
         <v>33</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D83" s="2">
         <v>0.38087534687534602</v>
@@ -3471,7 +3471,7 @@
         <v>34</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D84" s="2">
         <v>0.22279324652865501</v>
@@ -3500,7 +3500,7 @@
         <v>34</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D85" s="2">
         <v>0.38082931676739701</v>
@@ -3529,7 +3529,7 @@
         <v>11</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D86" s="2">
         <v>0.25720911168381899</v>
@@ -3558,7 +3558,7 @@
         <v>11</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D87" s="2">
         <v>0.37314315314315299</v>
@@ -3587,7 +3587,7 @@
         <v>13</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D88" s="2">
         <v>0.38501096926105699</v>
@@ -3616,7 +3616,7 @@
         <v>13</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D89" s="2">
         <v>0.38409896500805502</v>
@@ -3645,7 +3645,7 @@
         <v>15</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D90" s="2">
         <v>0.45806297424620701</v>
@@ -3674,7 +3674,7 @@
         <v>15</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D91" s="2">
         <v>0.39910165209016202</v>
@@ -3703,7 +3703,7 @@
         <v>22</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D92" s="3">
         <v>0.47648652687563198</v>
@@ -3732,7 +3732,7 @@
         <v>22</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D93" s="2">
         <v>0.40348660231969002</v>
@@ -3761,7 +3761,7 @@
         <v>29</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D94" s="2">
         <v>0.42238034879085401</v>
@@ -3790,7 +3790,7 @@
         <v>29</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D95" s="2">
         <v>0.45183195074846499</v>
@@ -3819,7 +3819,7 @@
         <v>0</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D96" s="2">
         <v>0.37932451249571802</v>
@@ -3848,7 +3848,7 @@
         <v>0</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D97" s="2">
         <v>0.44325601134637999</v>
@@ -3874,10 +3874,10 @@
         <v>2</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D98" s="2">
         <v>0.37287493127606303</v>
@@ -3903,10 +3903,10 @@
         <v>2</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D99" s="2">
         <v>0.158472591527927</v>
@@ -3935,7 +3935,7 @@
         <v>25</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D100" s="3">
         <v>3.6566662730232097E-2</v>
@@ -3964,7 +3964,7 @@
         <v>25</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D101" s="3">
         <v>6.88822715888429E-2</v>
@@ -3993,7 +3993,7 @@
         <v>12</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D102" s="3">
         <v>2.80388603725269E-2</v>
@@ -4022,7 +4022,7 @@
         <v>12</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D103" s="3">
         <v>5.8237537538380103E-2</v>
@@ -4051,7 +4051,7 @@
         <v>14</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D104" s="2">
         <v>0.10095224288789501</v>
@@ -4080,7 +4080,7 @@
         <v>14</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D105" s="2">
         <v>0.130638454310635</v>
@@ -4109,7 +4109,7 @@
         <v>16</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D106" s="3">
         <v>6.9187136825811998E-2</v>
@@ -4138,7 +4138,7 @@
         <v>16</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D107" s="2">
         <v>0.20137351824473701</v>
@@ -4167,7 +4167,7 @@
         <v>17</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D108" s="2">
         <v>0.119387158314899</v>
@@ -4196,7 +4196,7 @@
         <v>17</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D109" s="2">
         <v>0.26950973855510602</v>
@@ -4225,7 +4225,7 @@
         <v>18</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D110" s="2">
         <v>0.18152091034951301</v>
@@ -4254,7 +4254,7 @@
         <v>18</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D111" s="2">
         <v>0.272168043885609</v>
@@ -4283,7 +4283,7 @@
         <v>19</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D112" s="2">
         <v>0.216289083379855</v>
@@ -4312,7 +4312,7 @@
         <v>19</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D113" s="2">
         <v>0.31328423198503502</v>
@@ -4341,7 +4341,7 @@
         <v>20</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D114" s="2">
         <v>0.16748058955767001</v>
@@ -4370,7 +4370,7 @@
         <v>20</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D115" s="2">
         <v>0.271168766498604</v>
@@ -4399,7 +4399,7 @@
         <v>21</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D116" s="2">
         <v>0.19565688445763399</v>
@@ -4428,7 +4428,7 @@
         <v>21</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D117" s="2">
         <v>0.27582828326022701</v>
@@ -4457,7 +4457,7 @@
         <v>23</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D118" s="2">
         <v>0.25945260022950001</v>
@@ -4486,7 +4486,7 @@
         <v>23</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D119" s="2">
         <v>0.29497584265365601</v>
@@ -4515,7 +4515,7 @@
         <v>24</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D120" s="2">
         <v>0.232348379501603</v>
@@ -4544,7 +4544,7 @@
         <v>24</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D121" s="2">
         <v>0.28422210250922098</v>
@@ -4573,7 +4573,7 @@
         <v>26</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D122" s="2">
         <v>0.211239374036888</v>
@@ -4602,7 +4602,7 @@
         <v>26</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D123" s="2">
         <v>0.26740397078563999</v>
@@ -4631,7 +4631,7 @@
         <v>27</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D124" s="3">
         <v>0.22900078910807201</v>
@@ -4660,7 +4660,7 @@
         <v>27</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D125" s="2">
         <v>0.28869746609027902</v>
@@ -4689,7 +4689,7 @@
         <v>28</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D126" s="2">
         <v>0.224550184397493</v>
@@ -4718,7 +4718,7 @@
         <v>28</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D127" s="2">
         <v>0.27446932734068702</v>
@@ -4747,7 +4747,7 @@
         <v>30</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D128" s="2">
         <v>0.254032383767679</v>
@@ -4776,7 +4776,7 @@
         <v>30</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D129" s="3">
         <v>0.27703168733543299</v>
@@ -4805,7 +4805,7 @@
         <v>31</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D130" s="2">
         <v>0.22249503225641201</v>
@@ -4834,7 +4834,7 @@
         <v>31</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D131" s="2">
         <v>0.27740105621871802</v>
@@ -4863,7 +4863,7 @@
         <v>32</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D132" s="2">
         <v>0.245737577975913</v>
@@ -4892,7 +4892,7 @@
         <v>32</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D133" s="2">
         <v>0.27992907466237799</v>
@@ -4921,7 +4921,7 @@
         <v>33</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D134" s="2">
         <v>0.26446191025072502</v>
@@ -4950,7 +4950,7 @@
         <v>33</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D135" s="2">
         <v>0.27842357995237998</v>
@@ -4979,7 +4979,7 @@
         <v>34</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D136" s="2">
         <v>0.28781625247924503</v>
@@ -5008,7 +5008,7 @@
         <v>34</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D137" s="2">
         <v>0.284866566489762</v>
@@ -5037,7 +5037,7 @@
         <v>11</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D138" s="3">
         <v>0.246156426527358</v>
@@ -5066,7 +5066,7 @@
         <v>11</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D139" s="2">
         <v>0.27437864181376798</v>
@@ -5095,7 +5095,7 @@
         <v>13</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D140" s="2">
         <v>0.249786308374634</v>
@@ -5124,7 +5124,7 @@
         <v>13</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D141" s="3">
         <v>0.27177588112047601</v>
@@ -5153,7 +5153,7 @@
         <v>15</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D142" s="2">
         <v>0.192803138281474</v>
@@ -5182,7 +5182,7 @@
         <v>15</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D143" s="3">
         <v>0.27956944204794199</v>
@@ -5211,7 +5211,7 @@
         <v>22</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D144" s="2">
         <v>0.12916610488606101</v>
@@ -5240,7 +5240,7 @@
         <v>22</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D145" s="2">
         <v>0.29124817545443799</v>
@@ -5269,7 +5269,7 @@
         <v>29</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D146" s="2">
         <v>0.139602056204678</v>
@@ -5298,7 +5298,7 @@
         <v>29</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D147" s="3">
         <v>0.28323863418860301</v>
@@ -5327,7 +5327,7 @@
         <v>0</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D148" s="2">
         <v>0.102726035256184</v>
@@ -5356,7 +5356,7 @@
         <v>0</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D149" s="2">
         <v>0.268426728107934</v>
@@ -5382,10 +5382,10 @@
         <v>3</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D150" s="2">
         <v>0.13204993190754499</v>
@@ -5411,10 +5411,10 @@
         <v>3</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D151" s="2">
         <v>0.21610443213029301</v>
@@ -5443,7 +5443,7 @@
         <v>25</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D152" s="3">
         <v>1.37452997755734E-2</v>
@@ -5472,7 +5472,7 @@
         <v>25</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D153" s="3">
         <v>3.28041052067383E-2</v>
@@ -5501,7 +5501,7 @@
         <v>12</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D154" s="3">
         <v>1.5385627053076299E-2</v>
@@ -5530,7 +5530,7 @@
         <v>12</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D155" s="3">
         <v>5.7487100636436902E-2</v>
@@ -5559,7 +5559,7 @@
         <v>14</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D156" s="3">
         <v>2.0105050373956799E-2</v>
@@ -5588,7 +5588,7 @@
         <v>14</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D157" s="3">
         <v>7.6286660299473702E-2</v>
@@ -5617,7 +5617,7 @@
         <v>16</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D158" s="3">
         <v>2.5307809088267099E-2</v>
@@ -5646,7 +5646,7 @@
         <v>16</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D159" s="3">
         <v>8.5500974852427705E-2</v>
@@ -5675,7 +5675,7 @@
         <v>17</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D160" s="3">
         <v>3.54389799736365E-2</v>
@@ -5704,7 +5704,7 @@
         <v>17</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D161" s="3">
         <v>9.70473563705396E-2</v>
@@ -5733,7 +5733,7 @@
         <v>18</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D162" s="3">
         <v>3.55652500733937E-2</v>
@@ -5762,7 +5762,7 @@
         <v>18</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D163" s="2">
         <v>0.101013013315011</v>
@@ -5791,7 +5791,7 @@
         <v>19</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D164" s="3">
         <v>3.0365123156468901E-2</v>
@@ -5820,7 +5820,7 @@
         <v>19</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D165" s="2">
         <v>0.113205897190889</v>
@@ -5849,7 +5849,7 @@
         <v>20</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D166" s="3">
         <v>3.2557199921160997E-2</v>
@@ -5878,7 +5878,7 @@
         <v>20</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D167" s="3">
         <v>0.120387501430179</v>
@@ -5907,7 +5907,7 @@
         <v>21</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D168" s="3">
         <v>3.5705535241709802E-2</v>
@@ -5936,7 +5936,7 @@
         <v>21</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D169" s="2">
         <v>0.11606479750245099</v>
@@ -5965,7 +5965,7 @@
         <v>23</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D170" s="3">
         <v>3.61771318287058E-2</v>
@@ -5994,7 +5994,7 @@
         <v>23</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D171" s="2">
         <v>0.116525968878223</v>
@@ -6023,7 +6023,7 @@
         <v>24</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D172" s="3">
         <v>3.8615331454822002E-2</v>
@@ -6052,7 +6052,7 @@
         <v>24</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D173" s="2">
         <v>0.113158200829866</v>
@@ -6081,7 +6081,7 @@
         <v>26</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D174" s="3">
         <v>3.5204166531832899E-2</v>
@@ -6110,7 +6110,7 @@
         <v>26</v>
       </c>
       <c r="C175" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D175" s="2">
         <v>0.11733347279386599</v>
@@ -6139,7 +6139,7 @@
         <v>27</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D176" s="3">
         <v>3.7660640683075897E-2</v>
@@ -6168,7 +6168,7 @@
         <v>27</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D177" s="2">
         <v>0.115811588536333</v>
@@ -6197,7 +6197,7 @@
         <v>28</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D178" s="3">
         <v>3.80557404855877E-2</v>
@@ -6226,7 +6226,7 @@
         <v>28</v>
       </c>
       <c r="C179" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D179" s="2">
         <v>0.12040510920295699</v>
@@ -6255,7 +6255,7 @@
         <v>30</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D180" s="3">
         <v>4.1132288384849398E-2</v>
@@ -6284,7 +6284,7 @@
         <v>30</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D181" s="2">
         <v>0.113161454240828</v>
@@ -6313,7 +6313,7 @@
         <v>31</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D182" s="3">
         <v>3.7444479430596402E-2</v>
@@ -6342,7 +6342,7 @@
         <v>31</v>
       </c>
       <c r="C183" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D183" s="2">
         <v>0.117679660597374</v>
@@ -6371,7 +6371,7 @@
         <v>32</v>
       </c>
       <c r="C184" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D184" s="3">
         <v>3.78021059858199E-2</v>
@@ -6400,7 +6400,7 @@
         <v>32</v>
       </c>
       <c r="C185" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D185" s="3">
         <v>0.11985135916075</v>
@@ -6429,7 +6429,7 @@
         <v>33</v>
       </c>
       <c r="C186" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D186" s="3">
         <v>4.1126638640035601E-2</v>
@@ -6458,7 +6458,7 @@
         <v>33</v>
       </c>
       <c r="C187" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D187" s="2">
         <v>0.125016921765288</v>
@@ -6487,7 +6487,7 @@
         <v>34</v>
       </c>
       <c r="C188" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D188" s="3">
         <v>3.7089181503666697E-2</v>
@@ -6516,7 +6516,7 @@
         <v>34</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D189" s="2">
         <v>0.12704394619377299</v>
@@ -6545,7 +6545,7 @@
         <v>11</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D190" s="3">
         <v>3.5098217848716903E-2</v>
@@ -6574,7 +6574,7 @@
         <v>11</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D191" s="2">
         <v>0.12615485660893</v>
@@ -6603,7 +6603,7 @@
         <v>13</v>
       </c>
       <c r="C192" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D192" s="3">
         <v>2.9210450646463999E-2</v>
@@ -6632,7 +6632,7 @@
         <v>13</v>
       </c>
       <c r="C193" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D193" s="2">
         <v>0.13247458284473301</v>
@@ -6661,7 +6661,7 @@
         <v>15</v>
       </c>
       <c r="C194" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D194" s="3">
         <v>2.5084412243932101E-2</v>
@@ -6690,7 +6690,7 @@
         <v>15</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D195" s="2">
         <v>0.13382989222381</v>
@@ -6719,7 +6719,7 @@
         <v>22</v>
       </c>
       <c r="C196" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D196" s="3">
         <v>1.8219555961555198E-2</v>
@@ -6748,7 +6748,7 @@
         <v>22</v>
       </c>
       <c r="C197" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D197" s="2">
         <v>0.14254156408303001</v>
@@ -6777,7 +6777,7 @@
         <v>29</v>
       </c>
       <c r="C198" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D198" s="3">
         <v>1.9083149533110098E-2</v>
@@ -6806,7 +6806,7 @@
         <v>29</v>
       </c>
       <c r="C199" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D199" s="2">
         <v>0.165999726634388</v>
@@ -6835,7 +6835,7 @@
         <v>0</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D200" s="3">
         <v>1.9544483513473699E-2</v>
@@ -6864,7 +6864,7 @@
         <v>0</v>
       </c>
       <c r="C201" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D201" s="2">
         <v>0.17308994660476401</v>
@@ -6890,10 +6890,10 @@
         <v>4</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D202" s="3">
         <v>6.3453258388175393E-2</v>
@@ -6919,10 +6919,10 @@
         <v>4</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D203" s="2">
         <v>0.19480225822438901</v>
@@ -6951,7 +6951,7 @@
         <v>25</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D204" s="3">
         <v>6.3945067581989007E-2</v>
@@ -6980,7 +6980,7 @@
         <v>25</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D205" s="2">
         <v>0.101301553012049</v>
@@ -7009,7 +7009,7 @@
         <v>12</v>
       </c>
       <c r="C206" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D206" s="2">
         <v>0.14924208389583499</v>
@@ -7038,7 +7038,7 @@
         <v>12</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D207" s="2">
         <v>0.16595607406905299</v>
@@ -7067,7 +7067,7 @@
         <v>14</v>
       </c>
       <c r="C208" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D208" s="2">
         <v>0.26577151116457198</v>
@@ -7096,7 +7096,7 @@
         <v>14</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D209" s="2">
         <v>0.32749516939510198</v>
@@ -7125,7 +7125,7 @@
         <v>16</v>
       </c>
       <c r="C210" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D210" s="2">
         <v>0.32101640585785701</v>
@@ -7154,7 +7154,7 @@
         <v>16</v>
       </c>
       <c r="C211" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D211" s="2">
         <v>0.44994571492437802</v>
@@ -7183,7 +7183,7 @@
         <v>17</v>
       </c>
       <c r="C212" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D212" s="2">
         <v>0.347954493479114</v>
@@ -7212,7 +7212,7 @@
         <v>17</v>
       </c>
       <c r="C213" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D213" s="2">
         <v>0.46504472420810899</v>
@@ -7241,7 +7241,7 @@
         <v>18</v>
       </c>
       <c r="C214" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D214" s="2">
         <v>0.34163146216745399</v>
@@ -7270,7 +7270,7 @@
         <v>18</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D215" s="3">
         <v>0.47108737479908602</v>
@@ -7299,7 +7299,7 @@
         <v>19</v>
       </c>
       <c r="C216" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D216" s="2">
         <v>0.39538496841626902</v>
@@ -7328,7 +7328,7 @@
         <v>19</v>
       </c>
       <c r="C217" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D217" s="2">
         <v>0.506771290884239</v>
@@ -7357,7 +7357,7 @@
         <v>20</v>
       </c>
       <c r="C218" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D218" s="2">
         <v>0.39444082271569902</v>
@@ -7386,7 +7386,7 @@
         <v>20</v>
       </c>
       <c r="C219" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D219" s="2">
         <v>0.49232366114072201</v>
@@ -7415,7 +7415,7 @@
         <v>21</v>
       </c>
       <c r="C220" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D220" s="3">
         <v>0.37708398209744498</v>
@@ -7444,7 +7444,7 @@
         <v>21</v>
       </c>
       <c r="C221" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D221" s="3">
         <v>0.48613792891998697</v>
@@ -7473,7 +7473,7 @@
         <v>23</v>
       </c>
       <c r="C222" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D222" s="2">
         <v>0.37707936760442101</v>
@@ -7502,7 +7502,7 @@
         <v>23</v>
       </c>
       <c r="C223" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D223" s="2">
         <v>0.49892340369037202</v>
@@ -7531,7 +7531,7 @@
         <v>24</v>
       </c>
       <c r="C224" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D224" s="2">
         <v>0.36460396035176301</v>
@@ -7560,7 +7560,7 @@
         <v>24</v>
       </c>
       <c r="C225" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D225" s="2">
         <v>0.510846123904103</v>
@@ -7589,7 +7589,7 @@
         <v>26</v>
       </c>
       <c r="C226" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D226" s="2">
         <v>0.38387187139173901</v>
@@ -7618,7 +7618,7 @@
         <v>26</v>
       </c>
       <c r="C227" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D227" s="2">
         <v>0.50349585712525202</v>
@@ -7647,7 +7647,7 @@
         <v>27</v>
       </c>
       <c r="C228" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D228" s="2">
         <v>0.39751766601719302</v>
@@ -7676,7 +7676,7 @@
         <v>27</v>
       </c>
       <c r="C229" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D229" s="2">
         <v>0.51011586960372002</v>
@@ -7705,7 +7705,7 @@
         <v>28</v>
       </c>
       <c r="C230" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D230" s="2">
         <v>0.406406162390061</v>
@@ -7734,7 +7734,7 @@
         <v>28</v>
       </c>
       <c r="C231" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D231" s="2">
         <v>0.49829651498668698</v>
@@ -7763,7 +7763,7 @@
         <v>30</v>
       </c>
       <c r="C232" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D232" s="3">
         <v>0.40161883003674198</v>
@@ -7792,7 +7792,7 @@
         <v>30</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D233" s="2">
         <v>0.50951111793533799</v>
@@ -7821,7 +7821,7 @@
         <v>31</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D234" s="2">
         <v>0.431575938043948</v>
@@ -7850,7 +7850,7 @@
         <v>31</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D235" s="2">
         <v>0.50934004386293197</v>
@@ -7879,7 +7879,7 @@
         <v>32</v>
       </c>
       <c r="C236" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D236" s="2">
         <v>0.44908742210254698</v>
@@ -7908,7 +7908,7 @@
         <v>32</v>
       </c>
       <c r="C237" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D237" s="2">
         <v>0.50658110932299905</v>
@@ -7937,7 +7937,7 @@
         <v>33</v>
       </c>
       <c r="C238" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D238" s="2">
         <v>0.44714215033007199</v>
@@ -7966,7 +7966,7 @@
         <v>33</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D239" s="2">
         <v>0.51295619627903899</v>
@@ -7995,7 +7995,7 @@
         <v>34</v>
       </c>
       <c r="C240" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D240" s="2">
         <v>0.44116999357509601</v>
@@ -8024,7 +8024,7 @@
         <v>34</v>
       </c>
       <c r="C241" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D241" s="2">
         <v>0.51255060561374</v>
@@ -8053,7 +8053,7 @@
         <v>11</v>
       </c>
       <c r="C242" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D242" s="2">
         <v>0.43776154513256199</v>
@@ -8082,7 +8082,7 @@
         <v>11</v>
       </c>
       <c r="C243" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D243" s="2">
         <v>0.50287782257990399</v>
@@ -8111,7 +8111,7 @@
         <v>13</v>
       </c>
       <c r="C244" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D244" s="2">
         <v>0.45675918029513302</v>
@@ -8140,7 +8140,7 @@
         <v>13</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D245" s="2">
         <v>0.52258021411103905</v>
@@ -8169,7 +8169,7 @@
         <v>15</v>
       </c>
       <c r="C246" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D246" s="2">
         <v>0.45406791176268502</v>
@@ -8198,7 +8198,7 @@
         <v>15</v>
       </c>
       <c r="C247" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D247" s="2">
         <v>0.50860933469450798</v>
@@ -8227,7 +8227,7 @@
         <v>22</v>
       </c>
       <c r="C248" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D248" s="2">
         <v>0.46826829076068899</v>
@@ -8256,7 +8256,7 @@
         <v>22</v>
       </c>
       <c r="C249" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D249" s="2">
         <v>0.51569194056961898</v>
@@ -8285,7 +8285,7 @@
         <v>29</v>
       </c>
       <c r="C250" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D250" s="2">
         <v>0.48497358522769002</v>
@@ -8314,7 +8314,7 @@
         <v>29</v>
       </c>
       <c r="C251" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D251" s="2">
         <v>0.51276594049394797</v>
@@ -8343,7 +8343,7 @@
         <v>0</v>
       </c>
       <c r="C252" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D252" s="2">
         <v>0.47784246352508702</v>
@@ -8372,7 +8372,7 @@
         <v>0</v>
       </c>
       <c r="C253" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D253" s="2">
         <v>0.51981037485163495</v>
@@ -8398,10 +8398,10 @@
         <v>5</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C254" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D254" s="2">
         <v>0.43277780539543598</v>
@@ -8427,10 +8427,10 @@
         <v>5</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C255" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D255" s="2">
         <v>0.40733341662580003</v>
@@ -8459,7 +8459,7 @@
         <v>25</v>
       </c>
       <c r="C256" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D256" s="3">
         <v>8.0412703112476003E-3</v>
@@ -8488,7 +8488,7 @@
         <v>25</v>
       </c>
       <c r="C257" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D257" s="3">
         <v>8.8054854272070007E-3</v>
@@ -8517,7 +8517,7 @@
         <v>12</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D258" s="3">
         <v>6.8001888109682001E-3</v>
@@ -8546,7 +8546,7 @@
         <v>12</v>
       </c>
       <c r="C259" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D259" s="3">
         <v>9.0297463566422001E-3</v>
@@ -8575,7 +8575,7 @@
         <v>14</v>
       </c>
       <c r="C260" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D260" s="3">
         <v>7.9137702383727995E-3</v>
@@ -8604,7 +8604,7 @@
         <v>14</v>
       </c>
       <c r="C261" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D261" s="3">
         <v>1.0611184697368801E-2</v>
@@ -8633,7 +8633,7 @@
         <v>16</v>
       </c>
       <c r="C262" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D262" s="3">
         <v>7.5215875428721003E-3</v>
@@ -8662,7 +8662,7 @@
         <v>16</v>
       </c>
       <c r="C263" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D263" s="3">
         <v>4.4816747280090302E-2</v>
@@ -8691,7 +8691,7 @@
         <v>17</v>
       </c>
       <c r="C264" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D264" s="3">
         <v>7.5152368895052999E-3</v>
@@ -8720,7 +8720,7 @@
         <v>17</v>
       </c>
       <c r="C265" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D265" s="3">
         <v>3.5513286524182001E-2</v>
@@ -8749,7 +8749,7 @@
         <v>18</v>
       </c>
       <c r="C266" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D266" s="3">
         <v>7.5926334090982003E-3</v>
@@ -8778,7 +8778,7 @@
         <v>18</v>
       </c>
       <c r="C267" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D267" s="3">
         <v>3.2756303056082202E-2</v>
@@ -8807,7 +8807,7 @@
         <v>19</v>
       </c>
       <c r="C268" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D268" s="3">
         <v>1.0214644769684301E-2</v>
@@ -8836,7 +8836,7 @@
         <v>19</v>
       </c>
       <c r="C269" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D269" s="3">
         <v>3.9858266425174801E-2</v>
@@ -8865,7 +8865,7 @@
         <v>20</v>
       </c>
       <c r="C270" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D270" s="3">
         <v>1.5936086014944398E-2</v>
@@ -8894,7 +8894,7 @@
         <v>20</v>
       </c>
       <c r="C271" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D271" s="3">
         <v>5.0851862946548601E-2</v>
@@ -8923,7 +8923,7 @@
         <v>21</v>
       </c>
       <c r="C272" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D272" s="3">
         <v>2.9002794477229098E-2</v>
@@ -8952,7 +8952,7 @@
         <v>21</v>
       </c>
       <c r="C273" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D273" s="3">
         <v>5.5569042073598002E-2</v>
@@ -8981,7 +8981,7 @@
         <v>23</v>
       </c>
       <c r="C274" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D274" s="3">
         <v>2.88737973322498E-2</v>
@@ -9010,7 +9010,7 @@
         <v>23</v>
       </c>
       <c r="C275" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D275" s="3">
         <v>4.4493077115711897E-2</v>
@@ -9039,7 +9039,7 @@
         <v>24</v>
       </c>
       <c r="C276" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D276" s="3">
         <v>8.5692741677826395E-2</v>
@@ -9068,7 +9068,7 @@
         <v>24</v>
       </c>
       <c r="C277" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D277" s="3">
         <v>3.3631863297258403E-2</v>
@@ -9097,7 +9097,7 @@
         <v>26</v>
       </c>
       <c r="C278" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D278" s="3">
         <v>6.3976265056946993E-2</v>
@@ -9126,7 +9126,7 @@
         <v>26</v>
       </c>
       <c r="C279" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D279" s="3">
         <v>4.4426180511732798E-2</v>
@@ -9155,7 +9155,7 @@
         <v>27</v>
       </c>
       <c r="C280" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D280" s="3">
         <v>6.7140183732552705E-2</v>
@@ -9184,7 +9184,7 @@
         <v>27</v>
       </c>
       <c r="C281" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D281" s="3">
         <v>5.0552478650196297E-2</v>
@@ -9213,7 +9213,7 @@
         <v>28</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D282" s="3">
         <v>4.67239559902363E-2</v>
@@ -9242,7 +9242,7 @@
         <v>28</v>
       </c>
       <c r="C283" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D283" s="3">
         <v>6.44510393250146E-2</v>
@@ -9271,7 +9271,7 @@
         <v>30</v>
       </c>
       <c r="C284" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D284" s="3">
         <v>8.1986551309817204E-2</v>
@@ -9300,7 +9300,7 @@
         <v>30</v>
       </c>
       <c r="C285" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D285" s="3">
         <v>5.1290383472135298E-2</v>
@@ -9329,7 +9329,7 @@
         <v>31</v>
       </c>
       <c r="C286" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D286" s="3">
         <v>5.3241164777039399E-2</v>
@@ -9358,7 +9358,7 @@
         <v>31</v>
       </c>
       <c r="C287" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D287" s="3">
         <v>5.4345101459047397E-2</v>
@@ -9387,7 +9387,7 @@
         <v>32</v>
       </c>
       <c r="C288" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D288" s="3">
         <v>6.2478480820733602E-2</v>
@@ -9416,7 +9416,7 @@
         <v>32</v>
       </c>
       <c r="C289" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D289" s="3">
         <v>5.2698253820820502E-2</v>
@@ -9445,7 +9445,7 @@
         <v>33</v>
       </c>
       <c r="C290" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D290" s="3">
         <v>3.4731859185635101E-2</v>
@@ -9474,7 +9474,7 @@
         <v>33</v>
       </c>
       <c r="C291" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D291" s="3">
         <v>5.5528566039111001E-2</v>
@@ -9503,7 +9503,7 @@
         <v>34</v>
       </c>
       <c r="C292" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D292" s="3">
         <v>9.3736858636239706E-2</v>
@@ -9532,7 +9532,7 @@
         <v>34</v>
       </c>
       <c r="C293" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D293" s="3">
         <v>7.00311623912208E-2</v>
@@ -9561,7 +9561,7 @@
         <v>11</v>
       </c>
       <c r="C294" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D294" s="3">
         <v>5.99583213207096E-2</v>
@@ -9590,7 +9590,7 @@
         <v>11</v>
       </c>
       <c r="C295" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D295" s="3">
         <v>5.0107644782297199E-2</v>
@@ -9619,7 +9619,7 @@
         <v>13</v>
       </c>
       <c r="C296" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D296" s="3">
         <v>5.1857471026916201E-2</v>
@@ -9648,7 +9648,7 @@
         <v>13</v>
       </c>
       <c r="C297" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D297" s="3">
         <v>5.2863506715061903E-2</v>
@@ -9677,7 +9677,7 @@
         <v>15</v>
       </c>
       <c r="C298" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D298" s="3">
         <v>7.1133395491803905E-2</v>
@@ -9706,7 +9706,7 @@
         <v>15</v>
       </c>
       <c r="C299" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D299" s="3">
         <v>5.3073816098638198E-2</v>
@@ -9735,7 +9735,7 @@
         <v>22</v>
       </c>
       <c r="C300" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D300" s="3">
         <v>5.5011388313881998E-2</v>
@@ -9764,7 +9764,7 @@
         <v>22</v>
       </c>
       <c r="C301" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D301" s="3">
         <v>9.7393068118212398E-2</v>
@@ -9793,7 +9793,7 @@
         <v>29</v>
       </c>
       <c r="C302" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D302" s="3">
         <v>5.7309593406771601E-2</v>
@@ -9822,7 +9822,7 @@
         <v>29</v>
       </c>
       <c r="C303" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D303" s="2">
         <v>0.109903250829815</v>
@@ -9851,7 +9851,7 @@
         <v>0</v>
       </c>
       <c r="C304" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D304" s="3">
         <v>5.7474787574946097E-2</v>
@@ -9880,7 +9880,7 @@
         <v>0</v>
       </c>
       <c r="C305" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D305" s="3">
         <v>0.12380917128833099</v>
@@ -9906,10 +9906,10 @@
         <v>6</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C306" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D306" s="2">
         <v>0.108339813472301</v>
@@ -9935,10 +9935,10 @@
         <v>6</v>
       </c>
       <c r="B307" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C307" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D307" s="2">
         <v>0.177018916766949</v>
@@ -9967,7 +9967,7 @@
         <v>25</v>
       </c>
       <c r="C308" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D308" s="3">
         <v>7.1335927367054998E-3</v>
@@ -9996,7 +9996,7 @@
         <v>25</v>
       </c>
       <c r="C309" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D309" s="3">
         <v>8.6088154269972003E-3</v>
@@ -10025,7 +10025,7 @@
         <v>12</v>
       </c>
       <c r="C310" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D310" s="3">
         <v>7.1335927367054998E-3</v>
@@ -10054,7 +10054,7 @@
         <v>12</v>
       </c>
       <c r="C311" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D311" s="3">
         <v>8.6088154269972003E-3</v>
@@ -10083,7 +10083,7 @@
         <v>16</v>
       </c>
       <c r="C312" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D312" s="3">
         <v>1.75166118432056E-2</v>
@@ -10112,7 +10112,7 @@
         <v>16</v>
       </c>
       <c r="C313" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D313" s="3">
         <v>8.6088154269972003E-3</v>
@@ -10141,7 +10141,7 @@
         <v>18</v>
       </c>
       <c r="C314" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D314" s="3">
         <v>2.4287817420311199E-2</v>
@@ -10170,7 +10170,7 @@
         <v>18</v>
       </c>
       <c r="C315" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D315" s="3">
         <v>2.6635918769826499E-2</v>
@@ -10199,7 +10199,7 @@
         <v>20</v>
       </c>
       <c r="C316" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D316" s="3">
         <v>3.2945472425090702E-2</v>
@@ -10228,7 +10228,7 @@
         <v>20</v>
       </c>
       <c r="C317" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D317" s="3">
         <v>1.95172762232734E-2</v>
@@ -10257,7 +10257,7 @@
         <v>23</v>
       </c>
       <c r="C318" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D318" s="3">
         <v>5.5275910790750997E-2</v>
@@ -10286,7 +10286,7 @@
         <v>23</v>
       </c>
       <c r="C319" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D319" s="3">
         <v>1.8012130196057199E-2</v>
@@ -10315,7 +10315,7 @@
         <v>26</v>
       </c>
       <c r="C320" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D320" s="3">
         <v>4.0371634320198899E-2</v>
@@ -10344,7 +10344,7 @@
         <v>26</v>
       </c>
       <c r="C321" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D321" s="3">
         <v>1.5990811227610501E-2</v>
@@ -10373,7 +10373,7 @@
         <v>28</v>
       </c>
       <c r="C322" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D322" s="3">
         <v>2.68933899965129E-2</v>
@@ -10402,7 +10402,7 @@
         <v>28</v>
       </c>
       <c r="C323" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D323" s="3">
         <v>2.0558427273751699E-2</v>
@@ -10431,7 +10431,7 @@
         <v>31</v>
       </c>
       <c r="C324" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D324" s="3">
         <v>4.2294202330655603E-2</v>
@@ -10460,7 +10460,7 @@
         <v>31</v>
       </c>
       <c r="C325" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D325" s="3">
         <v>2.0897047531812301E-2</v>
@@ -10489,7 +10489,7 @@
         <v>33</v>
       </c>
       <c r="C326" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D326" s="3">
         <v>4.6211186078281001E-2</v>
@@ -10518,7 +10518,7 @@
         <v>33</v>
       </c>
       <c r="C327" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D327" s="3">
         <v>2.4114609850308898E-2</v>
@@ -10547,7 +10547,7 @@
         <v>11</v>
       </c>
       <c r="C328" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D328" s="3">
         <v>5.2125762992718899E-2</v>
@@ -10576,7 +10576,7 @@
         <v>11</v>
       </c>
       <c r="C329" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D329" s="3">
         <v>3.0563258178319098E-2</v>
@@ -10605,7 +10605,7 @@
         <v>13</v>
       </c>
       <c r="C330" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D330" s="3">
         <v>7.5540097908228798E-2</v>
@@ -10634,7 +10634,7 @@
         <v>13</v>
       </c>
       <c r="C331" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D331" s="3">
         <v>3.23422631473156E-2</v>
@@ -10663,7 +10663,7 @@
         <v>15</v>
       </c>
       <c r="C332" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D332" s="3">
         <v>5.18408431870023E-2</v>
@@ -10692,7 +10692,7 @@
         <v>15</v>
       </c>
       <c r="C333" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D333" s="3">
         <v>3.8139042345508099E-2</v>
@@ -10721,7 +10721,7 @@
         <v>22</v>
       </c>
       <c r="C334" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D334" s="3">
         <v>4.7921667382481901E-2</v>
@@ -10750,7 +10750,7 @@
         <v>22</v>
       </c>
       <c r="C335" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D335" s="3">
         <v>5.95908156182378E-2</v>
@@ -10779,7 +10779,7 @@
         <v>0</v>
       </c>
       <c r="C336" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D336" s="3">
         <v>4.8931525130854699E-2</v>
@@ -10808,7 +10808,7 @@
         <v>0</v>
       </c>
       <c r="C337" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D337" s="3">
         <v>7.1991464923364501E-2</v>
@@ -10837,7 +10837,7 @@
         <v>25</v>
       </c>
       <c r="C338" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D338" s="3">
         <v>1.5770103686068199E-2</v>
@@ -10866,7 +10866,7 @@
         <v>25</v>
       </c>
       <c r="C339" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D339" s="3">
         <v>1.48746162958057E-2</v>
@@ -10895,7 +10895,7 @@
         <v>12</v>
       </c>
       <c r="C340" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D340" s="3">
         <v>4.23117500240194E-2</v>
@@ -10924,7 +10924,7 @@
         <v>12</v>
       </c>
       <c r="C341" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D341" s="3">
         <v>4.0527995975801298E-2</v>
@@ -10953,7 +10953,7 @@
         <v>14</v>
       </c>
       <c r="C342" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D342" s="3">
         <v>4.7287720902358603E-2</v>
@@ -10982,7 +10982,7 @@
         <v>14</v>
       </c>
       <c r="C343" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D343" s="3">
         <v>3.56148764278333E-2</v>
@@ -11011,7 +11011,7 @@
         <v>16</v>
       </c>
       <c r="C344" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D344" s="3">
         <v>1.8554348106224101E-2</v>
@@ -11040,7 +11040,7 @@
         <v>16</v>
       </c>
       <c r="C345" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D345" s="3">
         <v>6.3342560264592701E-2</v>
@@ -11069,7 +11069,7 @@
         <v>17</v>
       </c>
       <c r="C346" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D346" s="3">
         <v>2.2911219248353099E-2</v>
@@ -11098,7 +11098,7 @@
         <v>17</v>
       </c>
       <c r="C347" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D347" s="3">
         <v>6.8291717176783506E-2</v>
@@ -11127,7 +11127,7 @@
         <v>18</v>
       </c>
       <c r="C348" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D348" s="3">
         <v>2.8104981151382099E-2</v>
@@ -11156,7 +11156,7 @@
         <v>18</v>
       </c>
       <c r="C349" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D349" s="3">
         <v>8.0465040431411394E-2</v>
@@ -11185,7 +11185,7 @@
         <v>19</v>
       </c>
       <c r="C350" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D350" s="3">
         <v>3.6603115452304602E-2</v>
@@ -11214,7 +11214,7 @@
         <v>19</v>
       </c>
       <c r="C351" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D351" s="3">
         <v>9.4445739776104404E-2</v>
@@ -11243,7 +11243,7 @@
         <v>20</v>
       </c>
       <c r="C352" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D352" s="3">
         <v>3.0618014199925901E-2</v>
@@ -11272,7 +11272,7 @@
         <v>20</v>
       </c>
       <c r="C353" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D353" s="3">
         <v>8.7797818443447195E-2</v>
@@ -11301,7 +11301,7 @@
         <v>21</v>
       </c>
       <c r="C354" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D354" s="3">
         <v>4.2675150751317302E-2</v>
@@ -11330,7 +11330,7 @@
         <v>21</v>
       </c>
       <c r="C355" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D355" s="3">
         <v>9.6024666923380006E-2</v>
@@ -11359,7 +11359,7 @@
         <v>23</v>
       </c>
       <c r="C356" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D356" s="3">
         <v>4.6011277993014799E-2</v>
@@ -11388,7 +11388,7 @@
         <v>23</v>
       </c>
       <c r="C357" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D357" s="3">
         <v>9.0166556422562397E-2</v>
@@ -11417,7 +11417,7 @@
         <v>24</v>
       </c>
       <c r="C358" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D358" s="3">
         <v>5.1861657964833101E-2</v>
@@ -11446,7 +11446,7 @@
         <v>24</v>
       </c>
       <c r="C359" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D359" s="2">
         <v>0.10176590820871</v>
@@ -11475,7 +11475,7 @@
         <v>26</v>
       </c>
       <c r="C360" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D360" s="3">
         <v>5.4532431435008598E-2</v>
@@ -11504,7 +11504,7 @@
         <v>26</v>
       </c>
       <c r="C361" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D361" s="3">
         <v>9.0730691519753506E-2</v>
@@ -11533,7 +11533,7 @@
         <v>27</v>
       </c>
       <c r="C362" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D362" s="3">
         <v>5.8067760202498098E-2</v>
@@ -11562,7 +11562,7 @@
         <v>27</v>
       </c>
       <c r="C363" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D363" s="3">
         <v>9.8284966693992504E-2</v>
@@ -11591,7 +11591,7 @@
         <v>28</v>
       </c>
       <c r="C364" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D364" s="3">
         <v>5.5083391817969701E-2</v>
@@ -11620,7 +11620,7 @@
         <v>28</v>
       </c>
       <c r="C365" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D365" s="3">
         <v>8.78040195143244E-2</v>
@@ -11649,7 +11649,7 @@
         <v>30</v>
       </c>
       <c r="C366" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D366" s="3">
         <v>5.77765138648135E-2</v>
@@ -11678,7 +11678,7 @@
         <v>30</v>
       </c>
       <c r="C367" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D367" s="3">
         <v>8.8884561618555097E-2</v>
@@ -11707,7 +11707,7 @@
         <v>31</v>
       </c>
       <c r="C368" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D368" s="3">
         <v>6.5020736385240002E-2</v>
@@ -11736,7 +11736,7 @@
         <v>31</v>
       </c>
       <c r="C369" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D369" s="3">
         <v>9.5162193513925505E-2</v>
@@ -11765,7 +11765,7 @@
         <v>32</v>
       </c>
       <c r="C370" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D370" s="3">
         <v>6.9346725429983394E-2</v>
@@ -11794,7 +11794,7 @@
         <v>32</v>
       </c>
       <c r="C371" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D371" s="3">
         <v>9.5458405300197099E-2</v>
@@ -11823,7 +11823,7 @@
         <v>33</v>
       </c>
       <c r="C372" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D372" s="3">
         <v>6.3660622953242499E-2</v>
@@ -11852,7 +11852,7 @@
         <v>33</v>
       </c>
       <c r="C373" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D373" s="3">
         <v>9.9178709094351294E-2</v>
@@ -11881,7 +11881,7 @@
         <v>34</v>
       </c>
       <c r="C374" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D374" s="3">
         <v>7.3931802559632998E-2</v>
@@ -11910,7 +11910,7 @@
         <v>34</v>
       </c>
       <c r="C375" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D375" s="3">
         <v>9.5577182505477601E-2</v>
@@ -11939,7 +11939,7 @@
         <v>11</v>
       </c>
       <c r="C376" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D376" s="3">
         <v>7.4507396921489596E-2</v>
@@ -11968,7 +11968,7 @@
         <v>11</v>
       </c>
       <c r="C377" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D377" s="3">
         <v>9.3876236909841204E-2</v>
@@ -11997,7 +11997,7 @@
         <v>13</v>
       </c>
       <c r="C378" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D378" s="3">
         <v>7.2520825598897207E-2</v>
@@ -12026,7 +12026,7 @@
         <v>13</v>
       </c>
       <c r="C379" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D379" s="2">
         <v>0.102596949120329</v>
@@ -12055,7 +12055,7 @@
         <v>15</v>
       </c>
       <c r="C380" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D380" s="3">
         <v>7.5523557938406205E-2</v>
@@ -12084,7 +12084,7 @@
         <v>15</v>
       </c>
       <c r="C381" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D381" s="2">
         <v>0.103063212078809</v>
@@ -12113,7 +12113,7 @@
         <v>22</v>
       </c>
       <c r="C382" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D382" s="3">
         <v>7.8629444879220897E-2</v>
@@ -12142,7 +12142,7 @@
         <v>22</v>
       </c>
       <c r="C383" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D383" s="2">
         <v>0.11368992309011999</v>
@@ -12171,7 +12171,7 @@
         <v>29</v>
       </c>
       <c r="C384" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D384" s="3">
         <v>5.91406466344487E-2</v>
@@ -12200,7 +12200,7 @@
         <v>29</v>
       </c>
       <c r="C385" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D385" s="2">
         <v>0.107202564320936</v>
@@ -12229,7 +12229,7 @@
         <v>0</v>
       </c>
       <c r="C386" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D386" s="3">
         <v>5.23910902775446E-2</v>
@@ -12258,7 +12258,7 @@
         <v>0</v>
       </c>
       <c r="C387" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D387" s="2">
         <v>0.107490497168633</v>
@@ -12284,10 +12284,10 @@
         <v>8</v>
       </c>
       <c r="B388" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C388" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D388" s="3">
         <v>6.1117537228431697E-2</v>
@@ -12313,10 +12313,10 @@
         <v>8</v>
       </c>
       <c r="B389" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C389" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D389" s="3">
         <v>5.6636074608452103E-2</v>
@@ -12345,7 +12345,7 @@
         <v>25</v>
       </c>
       <c r="C390" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D390" s="3">
         <v>1.6764261045299201E-2</v>
@@ -12374,7 +12374,7 @@
         <v>25</v>
       </c>
       <c r="C391" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D391" s="3">
         <v>1.1336143503418199E-2</v>
@@ -12403,7 +12403,7 @@
         <v>12</v>
       </c>
       <c r="C392" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D392" s="3">
         <v>1.5503233694579101E-2</v>
@@ -12432,7 +12432,7 @@
         <v>12</v>
       </c>
       <c r="C393" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D393" s="3">
         <v>1.8518754924874901E-2</v>
@@ -12461,7 +12461,7 @@
         <v>14</v>
       </c>
       <c r="C394" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D394" s="3">
         <v>2.348044374381E-2</v>
@@ -12490,7 +12490,7 @@
         <v>14</v>
       </c>
       <c r="C395" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D395" s="3">
         <v>2.72083982716687E-2</v>
@@ -12519,7 +12519,7 @@
         <v>16</v>
       </c>
       <c r="C396" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D396" s="3">
         <v>4.0505040738252097E-2</v>
@@ -12548,7 +12548,7 @@
         <v>16</v>
       </c>
       <c r="C397" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D397" s="3">
         <v>4.37518683483622E-2</v>
@@ -12577,7 +12577,7 @@
         <v>17</v>
       </c>
       <c r="C398" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D398" s="3">
         <v>6.0772293999215E-2</v>
@@ -12606,7 +12606,7 @@
         <v>17</v>
       </c>
       <c r="C399" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D399" s="3">
         <v>3.4951147731859998E-2</v>
@@ -12635,7 +12635,7 @@
         <v>18</v>
       </c>
       <c r="C400" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D400" s="3">
         <v>7.2729498432626494E-2</v>
@@ -12664,7 +12664,7 @@
         <v>18</v>
       </c>
       <c r="C401" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D401" s="3">
         <v>3.4500659455797E-2</v>
@@ -12693,7 +12693,7 @@
         <v>19</v>
       </c>
       <c r="C402" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D402" s="3">
         <v>9.3997583942050794E-2</v>
@@ -12722,7 +12722,7 @@
         <v>19</v>
       </c>
       <c r="C403" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D403" s="3">
         <v>3.7330892414672398E-2</v>
@@ -12751,7 +12751,7 @@
         <v>20</v>
       </c>
       <c r="C404" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D404" s="3">
         <v>8.2864249281233995E-2</v>
@@ -12780,7 +12780,7 @@
         <v>20</v>
       </c>
       <c r="C405" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D405" s="3">
         <v>3.42763041431315E-2</v>
@@ -12809,7 +12809,7 @@
         <v>21</v>
       </c>
       <c r="C406" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D406" s="3">
         <v>8.3803093301483597E-2</v>
@@ -12838,7 +12838,7 @@
         <v>21</v>
       </c>
       <c r="C407" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D407" s="3">
         <v>4.6765717339586697E-2</v>
@@ -12867,7 +12867,7 @@
         <v>23</v>
       </c>
       <c r="C408" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D408" s="3">
         <v>7.6895262596699196E-2</v>
@@ -12896,7 +12896,7 @@
         <v>23</v>
       </c>
       <c r="C409" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D409" s="3">
         <v>5.6846551502531602E-2</v>
@@ -12925,7 +12925,7 @@
         <v>24</v>
       </c>
       <c r="C410" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D410" s="2">
         <v>0.123298654768174</v>
@@ -12954,7 +12954,7 @@
         <v>24</v>
       </c>
       <c r="C411" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D411" s="3">
         <v>7.0971519691006305E-2</v>
@@ -12983,7 +12983,7 @@
         <v>26</v>
       </c>
       <c r="C412" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D412" s="3">
         <v>0.105969872768028</v>
@@ -13012,7 +13012,7 @@
         <v>26</v>
       </c>
       <c r="C413" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D413" s="3">
         <v>5.8090720790113397E-2</v>
@@ -13041,7 +13041,7 @@
         <v>27</v>
       </c>
       <c r="C414" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D414" s="2">
         <v>0.1454572537272</v>
@@ -13070,7 +13070,7 @@
         <v>27</v>
       </c>
       <c r="C415" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D415" s="3">
         <v>6.3668538469361199E-2</v>
@@ -13099,7 +13099,7 @@
         <v>28</v>
       </c>
       <c r="C416" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D416" s="2">
         <v>0.122791795505347</v>
@@ -13128,7 +13128,7 @@
         <v>28</v>
       </c>
       <c r="C417" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D417" s="3">
         <v>6.2754226728284304E-2</v>
@@ -13157,7 +13157,7 @@
         <v>30</v>
       </c>
       <c r="C418" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D418" s="2">
         <v>0.135923149036625</v>
@@ -13186,7 +13186,7 @@
         <v>30</v>
       </c>
       <c r="C419" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D419" s="3">
         <v>5.4764418498985702E-2</v>
@@ -13215,7 +13215,7 @@
         <v>31</v>
       </c>
       <c r="C420" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D420" s="2">
         <v>0.10773438859532899</v>
@@ -13244,7 +13244,7 @@
         <v>31</v>
       </c>
       <c r="C421" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D421" s="3">
         <v>5.4352590581292402E-2</v>
@@ -13273,7 +13273,7 @@
         <v>32</v>
       </c>
       <c r="C422" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D422" s="2">
         <v>0.103921292579427</v>
@@ -13302,7 +13302,7 @@
         <v>32</v>
       </c>
       <c r="C423" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D423" s="3">
         <v>6.1949704182393303E-2</v>
@@ -13331,7 +13331,7 @@
         <v>33</v>
       </c>
       <c r="C424" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D424" s="2">
         <v>0.13109413591149599</v>
@@ -13360,7 +13360,7 @@
         <v>33</v>
       </c>
       <c r="C425" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D425" s="3">
         <v>6.57042766731116E-2</v>
@@ -13389,7 +13389,7 @@
         <v>34</v>
       </c>
       <c r="C426" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D426" s="2">
         <v>0.114911306702097</v>
@@ -13418,7 +13418,7 @@
         <v>34</v>
       </c>
       <c r="C427" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D427" s="3">
         <v>6.4900542709569006E-2</v>
@@ -13447,7 +13447,7 @@
         <v>11</v>
       </c>
       <c r="C428" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D428" s="2">
         <v>0.137394471383261</v>
@@ -13476,7 +13476,7 @@
         <v>11</v>
       </c>
       <c r="C429" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D429" s="3">
         <v>7.2061365166561905E-2</v>
@@ -13505,7 +13505,7 @@
         <v>13</v>
       </c>
       <c r="C430" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D430" s="2">
         <v>0.135016004885612</v>
@@ -13534,7 +13534,7 @@
         <v>13</v>
       </c>
       <c r="C431" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D431" s="3">
         <v>7.6008811644355606E-2</v>
@@ -13563,7 +13563,7 @@
         <v>15</v>
       </c>
       <c r="C432" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D432" s="3">
         <v>9.7389881514657994E-2</v>
@@ -13592,7 +13592,7 @@
         <v>15</v>
       </c>
       <c r="C433" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D433" s="3">
         <v>6.3735713417533604E-2</v>
@@ -13621,7 +13621,7 @@
         <v>22</v>
       </c>
       <c r="C434" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D434" s="3">
         <v>8.9604839971147807E-2</v>
@@ -13650,7 +13650,7 @@
         <v>22</v>
       </c>
       <c r="C435" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D435" s="3">
         <v>9.0687515576045805E-2</v>
@@ -13679,7 +13679,7 @@
         <v>29</v>
       </c>
       <c r="C436" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D436" s="3">
         <v>8.8615284773496894E-2</v>
@@ -13708,7 +13708,7 @@
         <v>29</v>
       </c>
       <c r="C437" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D437" s="3">
         <v>8.6870676200065403E-2</v>
@@ -13737,7 +13737,7 @@
         <v>0</v>
       </c>
       <c r="C438" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D438" s="3">
         <v>9.9138072796877405E-2</v>
@@ -13766,7 +13766,7 @@
         <v>0</v>
       </c>
       <c r="C439" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D439" s="3">
         <v>7.3420783629369907E-2</v>
@@ -13792,10 +13792,10 @@
         <v>9</v>
       </c>
       <c r="B440" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C440" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D440" s="3">
         <v>7.7781781808831496E-2</v>
@@ -13821,10 +13821,10 @@
         <v>9</v>
       </c>
       <c r="B441" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C441" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D441" s="3">
         <v>2.0279112561891698E-2</v>
@@ -13853,7 +13853,7 @@
         <v>16</v>
       </c>
       <c r="C442" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D442" s="3">
         <v>8.6088154269972003E-3</v>
@@ -13878,7 +13878,7 @@
         <v>17</v>
       </c>
       <c r="C443" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D443" s="3">
         <v>8.6088154269972003E-3</v>
@@ -13903,7 +13903,7 @@
         <v>18</v>
       </c>
       <c r="C444" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D444" s="3">
         <v>2.8264462809917301E-2</v>
@@ -13932,7 +13932,7 @@
         <v>19</v>
       </c>
       <c r="C445" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D445" s="3">
         <v>7.1335927367054998E-3</v>
@@ -13957,7 +13957,7 @@
         <v>19</v>
       </c>
       <c r="C446" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D446" s="3">
         <v>1.8436639118457301E-2</v>
@@ -13986,7 +13986,7 @@
         <v>20</v>
       </c>
       <c r="C447" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D447" s="3">
         <v>5.2263883975946203E-2</v>
@@ -14015,7 +14015,7 @@
         <v>20</v>
       </c>
       <c r="C448" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D448" s="3">
         <v>2.1827364554637199E-2</v>
@@ -14044,7 +14044,7 @@
         <v>21</v>
       </c>
       <c r="C449" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D449" s="3">
         <v>6.7307314389026401E-2</v>
@@ -14073,7 +14073,7 @@
         <v>21</v>
       </c>
       <c r="C450" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D450" s="3">
         <v>3.5883510428964899E-2</v>
@@ -14102,7 +14102,7 @@
         <v>23</v>
       </c>
       <c r="C451" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D451" s="3">
         <v>5.2263883975946203E-2</v>
@@ -14131,7 +14131,7 @@
         <v>23</v>
       </c>
       <c r="C452" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D452" s="3">
         <v>5.1356017719654E-2</v>
@@ -14160,7 +14160,7 @@
         <v>24</v>
       </c>
       <c r="C453" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D453" s="3">
         <v>6.7307314389026401E-2</v>
@@ -14189,7 +14189,7 @@
         <v>24</v>
       </c>
       <c r="C454" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D454" s="3">
         <v>7.4357150594735105E-2</v>
@@ -14218,7 +14218,7 @@
         <v>26</v>
       </c>
       <c r="C455" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D455" s="3">
         <v>7.1753149574161207E-2</v>
@@ -14247,7 +14247,7 @@
         <v>26</v>
       </c>
       <c r="C456" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D456" s="3">
         <v>4.9161775820160902E-2</v>
@@ -14276,7 +14276,7 @@
         <v>27</v>
       </c>
       <c r="C457" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D457" s="3">
         <v>5.3577631398643001E-2</v>
@@ -14305,7 +14305,7 @@
         <v>27</v>
       </c>
       <c r="C458" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D458" s="3">
         <v>6.1054178798384297E-2</v>
@@ -14334,7 +14334,7 @@
         <v>28</v>
       </c>
       <c r="C459" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D459" s="3">
         <v>3.92760481315425E-2</v>
@@ -14363,7 +14363,7 @@
         <v>28</v>
       </c>
       <c r="C460" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D460" s="3">
         <v>5.6354570898735502E-2</v>
@@ -14392,7 +14392,7 @@
         <v>30</v>
       </c>
       <c r="C461" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D461" s="3">
         <v>6.9619507591583502E-2</v>
@@ -14421,7 +14421,7 @@
         <v>30</v>
       </c>
       <c r="C462" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D462" s="3">
         <v>6.6843680156002297E-2</v>
@@ -14450,7 +14450,7 @@
         <v>31</v>
       </c>
       <c r="C463" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D463" s="3">
         <v>9.9601664672600398E-2</v>
@@ -14479,7 +14479,7 @@
         <v>31</v>
       </c>
       <c r="C464" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D464" s="3">
         <v>7.6958652514171805E-2</v>
@@ -14508,7 +14508,7 @@
         <v>32</v>
       </c>
       <c r="C465" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D465" s="3">
         <v>6.9723744933336204E-2</v>
@@ -14537,7 +14537,7 @@
         <v>32</v>
       </c>
       <c r="C466" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D466" s="3">
         <v>0.14094099474583099</v>
@@ -14566,7 +14566,7 @@
         <v>33</v>
       </c>
       <c r="C467" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D467" s="2">
         <v>0.13172257224824399</v>
@@ -14595,7 +14595,7 @@
         <v>33</v>
       </c>
       <c r="C468" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D468" s="3">
         <v>8.5473612941882396E-2</v>
@@ -14624,7 +14624,7 @@
         <v>34</v>
       </c>
       <c r="C469" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D469" s="3">
         <v>8.4743695255427298E-2</v>
@@ -14653,7 +14653,7 @@
         <v>34</v>
       </c>
       <c r="C470" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D470" s="3">
         <v>8.9580422836612605E-2</v>
@@ -14682,7 +14682,7 @@
         <v>11</v>
       </c>
       <c r="C471" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D471" s="3">
         <v>8.4136833325460805E-2</v>
@@ -14711,7 +14711,7 @@
         <v>11</v>
       </c>
       <c r="C472" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D472" s="3">
         <v>7.7138065334217201E-2</v>
@@ -14740,7 +14740,7 @@
         <v>13</v>
       </c>
       <c r="C473" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D473" s="3">
         <v>4.8284513292827201E-2</v>
@@ -14769,7 +14769,7 @@
         <v>13</v>
       </c>
       <c r="C474" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D474" s="3">
         <v>4.2330839014296497E-2</v>
@@ -14798,7 +14798,7 @@
         <v>15</v>
       </c>
       <c r="C475" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D475" s="3">
         <v>3.9782926918211801E-2</v>
@@ -14827,7 +14827,7 @@
         <v>15</v>
       </c>
       <c r="C476" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D476" s="3">
         <v>9.6353720611959001E-2</v>
@@ -14856,7 +14856,7 @@
         <v>22</v>
       </c>
       <c r="C477" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D477" s="3">
         <v>5.5118201112023701E-2</v>
@@ -14885,7 +14885,7 @@
         <v>22</v>
       </c>
       <c r="C478" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D478" s="2">
         <v>0.112693670419824</v>
@@ -14914,7 +14914,7 @@
         <v>29</v>
       </c>
       <c r="C479" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D479" s="3">
         <v>6.12244519800079E-2</v>
@@ -14943,7 +14943,7 @@
         <v>29</v>
       </c>
       <c r="C480" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D480" s="2">
         <v>0.11943579701291</v>
@@ -14972,7 +14972,7 @@
         <v>0</v>
       </c>
       <c r="C481" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D481" s="3">
         <v>8.0238467099157704E-2</v>
@@ -15001,7 +15001,7 @@
         <v>0</v>
       </c>
       <c r="C482" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D482" s="2">
         <v>0.107715165171424</v>
@@ -15027,10 +15027,10 @@
         <v>10</v>
       </c>
       <c r="B483" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C483" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D483" s="2">
         <v>0.159800566156024</v>
@@ -15056,10 +15056,10 @@
         <v>10</v>
       </c>
       <c r="B484" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C484" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D484" s="3">
         <v>7.0857820520816794E-2</v>

</xml_diff>